<commit_message>
Add Tab 3: passport label + photo sheet generator
</commit_message>
<xml_diff>
--- a/passengers.xlsx
+++ b/passengers.xlsx
@@ -35,7 +35,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +45,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,10 +79,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -447,12 +455,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,55 +482,719 @@
           <t>passport</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>นาย สมชาย ใจดี</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Mr. Somchai Jaidee</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>AA1234567</t>
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>S__1015816_0.jpg</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>นางสาว มาลี รักเรียน</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Ms. Malee Rakrian</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>BB7654321</t>
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>S__1015819_0.jpg</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>เด็กชาย ก้อง แก้วใส</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Master Kong Kaewsai</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>CC1112223</t>
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>S__1015822_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>S__1015825_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>S__1015831_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>S__1015834_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>S__1015837_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>S__1015840_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>S__1015843_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>S__1015846_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>S__1015849.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>S__1015852_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>S__1015855.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>S__1015858_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>S__1015861_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>S__1015864_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>S__1015867_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>S__1015870_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>S__1015873_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>S__1015876_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>S__1015879_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>S__1015882_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>S__1015885_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>S__1015888_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>S__1015891_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>S__1015897_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>S__1015900_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>S__1015903_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>S__1024005_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>S__1024008_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>S__1064965.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>S__1064968.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>S__1064971_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>S__1064974_0.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr"/>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>gemini</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>เรียก Gemini ไม่สำเร็จ: gemini-1.5-flash: 404 models/gemini-1.5-flash is not found for API version v1beta, or is not supported for generateContent. Call ModelService.ListModels to see the list of available models and their supported methods.</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>S__1138696.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>